<commit_message>
Update Naruto tier list again (78 -> 62) + cache-bust character data
Regenerated characters.json from the latest spreadsheet edit. Also
added a DATA_VERSION-based cache-busting query param on the
characters.json fetch, since GitHub Pages caches static files for
~10 minutes and each tier-list update was showing stale counts on
first load until that window expired. Bump DATA_VERSION in app.js
whenever data/characters.json is regenerated going forward so updates
go out immediately.
</commit_message>
<xml_diff>
--- a/sources/tier_list_naruto_2.xlsx
+++ b/sources/tier_list_naruto_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaisonramos/Documents/Claude/JeuxTiktok/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3D5AAC3-0F7E-D24B-A9E4-D8FD37422059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36442A6-94DE-E240-8D69-25EB1341CF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="16380" windowHeight="8200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier List" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Doublons retires" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tier List'!$A$1:$D$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tier List'!$A$1:$D$65</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="93">
   <si>
     <t>Rang</t>
   </si>
@@ -79,12 +79,6 @@
     <t>Six Paths</t>
   </si>
   <si>
-    <t>Ashura</t>
-  </si>
-  <si>
-    <t>Indra</t>
-  </si>
-  <si>
     <t>Kakashi</t>
   </si>
   <si>
@@ -136,12 +130,6 @@
     <t>Killer Bee</t>
   </si>
   <si>
-    <t>Lord Mu</t>
-  </si>
-  <si>
-    <t>Gengetsu</t>
-  </si>
-  <si>
     <t>Onoki</t>
   </si>
   <si>
@@ -160,9 +148,6 @@
     <t>White Zetsu</t>
   </si>
   <si>
-    <t>Sakumo</t>
-  </si>
-  <si>
     <t>Tsunade</t>
   </si>
   <si>
@@ -205,9 +190,6 @@
     <t>Deidara</t>
   </si>
   <si>
-    <t>Rasa</t>
-  </si>
-  <si>
     <t>Choji</t>
   </si>
   <si>
@@ -220,24 +202,12 @@
     <t>Rock Lee</t>
   </si>
   <si>
-    <t>Fugaku</t>
-  </si>
-  <si>
     <t>Kage Level Contenders</t>
   </si>
   <si>
-    <t>Yugito</t>
-  </si>
-  <si>
-    <t>Darui</t>
-  </si>
-  <si>
     <t>Kinkaku / Ginkaku</t>
   </si>
   <si>
-    <t>Mifune</t>
-  </si>
-  <si>
     <t>Tenten</t>
   </si>
   <si>
@@ -265,9 +235,6 @@
     <t>Kankuro</t>
   </si>
   <si>
-    <t>Fu / Torune</t>
-  </si>
-  <si>
     <t>Yamato</t>
   </si>
   <si>
@@ -280,12 +247,6 @@
     <t>Suigetsu</t>
   </si>
   <si>
-    <t>Chojuro</t>
-  </si>
-  <si>
-    <t>Jugo</t>
-  </si>
-  <si>
     <t>Kurenai</t>
   </si>
   <si>
@@ -311,15 +272,6 @@
   </si>
   <si>
     <t>Akatsuchi</t>
-  </si>
-  <si>
-    <t>Aoba</t>
-  </si>
-  <si>
-    <t>Genma</t>
-  </si>
-  <si>
-    <t>Anko</t>
   </si>
   <si>
     <t>Shizune</t>
@@ -841,7 +793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -959,46 +911,46 @@
         <v>12</v>
       </c>
       <c r="D8" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>2</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>11</v>
+      <c r="B9" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D9" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>2</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>11</v>
+        <v>3</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>15</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D10" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>3</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>15</v>
+        <v>4</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>17</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D11" s="2">
         <v>1</v>
@@ -1006,13 +958,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>4</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>17</v>
+        <v>5</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D12" s="2">
         <v>1</v>
@@ -1020,13 +972,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>5</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>19</v>
+        <v>6</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>21</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D13" s="2">
         <v>1</v>
@@ -1036,25 +988,25 @@
       <c r="A14" s="2">
         <v>6</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D14" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>7</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>23</v>
+        <v>8</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>24</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D15" s="2">
         <v>1</v>
@@ -1062,13 +1014,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>7</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>23</v>
+        <v>8</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>24</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D16" s="2">
         <v>2</v>
@@ -1079,13 +1031,13 @@
         <v>8</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -1093,13 +1045,13 @@
         <v>8</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D18" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -1107,13 +1059,13 @@
         <v>8</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>29</v>
       </c>
       <c r="D19" s="2">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -1121,13 +1073,13 @@
         <v>8</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D20" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -1135,13 +1087,13 @@
         <v>8</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>31</v>
       </c>
       <c r="D21" s="2">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -1149,69 +1101,69 @@
         <v>8</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>32</v>
       </c>
       <c r="D22" s="2">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>8</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>26</v>
+        <v>9</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>33</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D23" s="2">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>8</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>26</v>
+        <v>9</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>33</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D24" s="2">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>8</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>26</v>
+        <v>9</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>33</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D25" s="2">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>8</v>
-      </c>
-      <c r="B26" s="11" t="s">
-        <v>26</v>
+        <v>9</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>33</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D26" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -1219,13 +1171,13 @@
         <v>9</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D27" s="2">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -1233,13 +1185,13 @@
         <v>9</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>39</v>
       </c>
       <c r="D28" s="2">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -1247,13 +1199,13 @@
         <v>9</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>40</v>
       </c>
       <c r="D29" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -1261,13 +1213,13 @@
         <v>9</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>41</v>
       </c>
       <c r="D30" s="2">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -1275,83 +1227,83 @@
         <v>9</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D31" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>9</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>43</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D32" s="2">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>9</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>43</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D33" s="2">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>9</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>43</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D34" s="2">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>9</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>43</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D35" s="2">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>9</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>43</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D36" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
@@ -1359,13 +1311,13 @@
         <v>10</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>49</v>
       </c>
       <c r="D37" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -1373,13 +1325,13 @@
         <v>10</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>50</v>
       </c>
       <c r="D38" s="2">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
@@ -1387,13 +1339,13 @@
         <v>10</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>51</v>
       </c>
       <c r="D39" s="2">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
@@ -1401,248 +1353,248 @@
         <v>10</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>52</v>
       </c>
       <c r="D40" s="2">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>10</v>
-      </c>
-      <c r="B41" s="13" t="s">
-        <v>48</v>
+        <v>11</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>53</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D41" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>10</v>
-      </c>
-      <c r="B42" s="13" t="s">
-        <v>48</v>
+        <v>11</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>53</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D42" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>10</v>
-      </c>
-      <c r="B43" s="13" t="s">
-        <v>48</v>
+        <v>11</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>53</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D43" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>10</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>48</v>
+        <v>11</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>53</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D44" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>10</v>
-      </c>
-      <c r="B45" s="13" t="s">
-        <v>48</v>
+        <v>11</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>53</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D45" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
-        <v>10</v>
-      </c>
-      <c r="B46" s="13" t="s">
-        <v>48</v>
+        <v>12</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D46" s="2">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
-        <v>10</v>
-      </c>
-      <c r="B47" s="13" t="s">
-        <v>48</v>
+        <v>12</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D47" s="2">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
-        <v>11</v>
-      </c>
-      <c r="B48" s="14" t="s">
-        <v>60</v>
+        <v>12</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D48" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
-        <v>11</v>
-      </c>
-      <c r="B49" s="14" t="s">
-        <v>60</v>
+        <v>12</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D49" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
-        <v>11</v>
-      </c>
-      <c r="B50" s="14" t="s">
-        <v>60</v>
+        <v>12</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D50" s="2">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
-        <v>11</v>
-      </c>
-      <c r="B51" s="14" t="s">
-        <v>60</v>
+        <v>12</v>
+      </c>
+      <c r="B51" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D51" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
-        <v>11</v>
-      </c>
-      <c r="B52" s="14" t="s">
-        <v>60</v>
+        <v>12</v>
+      </c>
+      <c r="B52" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D52" s="2">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
-        <v>11</v>
-      </c>
-      <c r="B53" s="14" t="s">
-        <v>60</v>
+        <v>12</v>
+      </c>
+      <c r="B53" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D53" s="2">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
-        <v>11</v>
-      </c>
-      <c r="B54" s="14" t="s">
-        <v>60</v>
+        <v>12</v>
+      </c>
+      <c r="B54" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D54" s="2">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
-        <v>11</v>
-      </c>
-      <c r="B55" s="14" t="s">
-        <v>60</v>
+        <v>13</v>
+      </c>
+      <c r="B55" s="16" t="s">
+        <v>69</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D55" s="2">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
-        <v>12</v>
-      </c>
-      <c r="B56" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B56" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D56" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
-        <v>12</v>
-      </c>
-      <c r="B57" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B57" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D57" s="2">
         <v>3</v>
@@ -1650,13 +1602,13 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
-        <v>12</v>
-      </c>
-      <c r="B58" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B58" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D58" s="2">
         <v>4</v>
@@ -1664,13 +1616,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
-        <v>12</v>
-      </c>
-      <c r="B59" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B59" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D59" s="2">
         <v>5</v>
@@ -1678,13 +1630,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
-        <v>12</v>
-      </c>
-      <c r="B60" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D60" s="2">
         <v>6</v>
@@ -1692,13 +1644,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
-        <v>12</v>
-      </c>
-      <c r="B61" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D61" s="2">
         <v>7</v>
@@ -1706,258 +1658,34 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
-        <v>12</v>
-      </c>
-      <c r="B62" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B62" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D62" s="2">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="2">
-        <v>12</v>
-      </c>
-      <c r="B63" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B63" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D63" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="2">
-        <v>12</v>
-      </c>
-      <c r="B64" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C64" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D64" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="2">
-        <v>12</v>
-      </c>
-      <c r="B65" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D65" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="2">
-        <v>12</v>
-      </c>
-      <c r="B66" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D66" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="2">
-        <v>12</v>
-      </c>
-      <c r="B67" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D67" s="2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="2">
-        <v>13</v>
-      </c>
-      <c r="B68" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D68" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="2">
-        <v>13</v>
-      </c>
-      <c r="B69" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D69" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="2">
-        <v>13</v>
-      </c>
-      <c r="B70" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D70" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="2">
-        <v>13</v>
-      </c>
-      <c r="B71" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D71" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="2">
-        <v>13</v>
-      </c>
-      <c r="B72" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C72" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D72" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="2">
-        <v>13</v>
-      </c>
-      <c r="B73" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C73" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D73" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="2">
-        <v>13</v>
-      </c>
-      <c r="B74" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D74" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="2">
-        <v>13</v>
-      </c>
-      <c r="B75" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C75" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D75" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="2">
-        <v>13</v>
-      </c>
-      <c r="B76" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D76" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="2">
-        <v>13</v>
-      </c>
-      <c r="B77" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C77" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D77" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="2">
-        <v>13</v>
-      </c>
-      <c r="B78" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D78" s="2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="2">
-        <v>13</v>
-      </c>
-      <c r="B79" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D79" s="2">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D91" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:D77" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1981,7 +1709,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -2005,7 +1733,7 @@
       </c>
       <c r="C3" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B3)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2013,7 +1741,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B4)</f>
@@ -2025,7 +1753,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B5)</f>
@@ -2037,7 +1765,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B6)</f>
@@ -2049,7 +1777,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B7)</f>
@@ -2061,7 +1789,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B8)</f>
@@ -2073,11 +1801,11 @@
         <v>8</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B9)</f>
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -2085,11 +1813,11 @@
         <v>9</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C10" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B10)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -2097,11 +1825,11 @@
         <v>10</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C11" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B11)</f>
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2109,11 +1837,11 @@
         <v>11</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B12)</f>
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -2121,11 +1849,11 @@
         <v>12</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B13)</f>
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -2133,11 +1861,11 @@
         <v>13</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B14)</f>
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -2145,7 +1873,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B15)</f>
@@ -2157,7 +1885,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C16" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B16)</f>
@@ -2169,7 +1897,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C17" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B17)</f>
@@ -2181,7 +1909,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C18" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B18)</f>
@@ -2193,7 +1921,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="C19" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B19)</f>
@@ -2205,7 +1933,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C20" s="2">
         <f>COUNTIF('Tier List'!$B:$B,B20)</f>
@@ -2214,16 +1942,16 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B21" s="21" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C21" s="22">
         <f>SUM(C2:C20)</f>
-        <v>78</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="23" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2246,7 +1974,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -2294,7 +2022,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -2302,15 +2030,15 @@
         <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -2318,7 +2046,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -2326,7 +2054,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -2334,15 +2062,15 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -2350,7 +2078,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -2358,7 +2086,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -2366,47 +2094,47 @@
         <v>8</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -2414,15 +2142,15 @@
         <v>8</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
@@ -2430,15 +2158,15 @@
         <v>9</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -2446,15 +2174,15 @@
         <v>8</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -2462,87 +2190,87 @@
         <v>9</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -2550,23 +2278,23 @@
         <v>9</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -2574,23 +2302,23 @@
         <v>8</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -2598,39 +2326,39 @@
         <v>8</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -2638,7 +2366,7 @@
         <v>9</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
@@ -2646,31 +2374,31 @@
         <v>8</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
@@ -2678,7 +2406,7 @@
         <v>9</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
@@ -2686,63 +2414,63 @@
         <v>8</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
@@ -2750,39 +2478,39 @@
         <v>9</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
@@ -2790,31 +2518,31 @@
         <v>9</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>